<commit_message>
static 제거 Excel 에 st_STC_AoiInPlayerMoves 추가
</commit_message>
<xml_diff>
--- a/WRExcel/RPC_GAME_EXCEL.xlsx
+++ b/WRExcel/RPC_GAME_EXCEL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WRExcel\WRExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B0BA71-BEBE-4F39-8961-0C286A8F4904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42DB1F8-9B84-45D9-8827-BD3CF3A88B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35210" yWindow="4940" windowWidth="28800" windowHeight="15460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32910" yWindow="3120" windowWidth="28800" windowHeight="15460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Struct" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="132">
   <si>
     <t>NULL</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -532,6 +532,26 @@
   </si>
   <si>
     <t>st_STC_OtherMoveStart</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>st_PlayerOtherMove</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AOI_IN_PLAYERS_MOVE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>st_STC_AoiInPlayerMoves</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>move[50]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AOI 안에 들어온 Player Move 패킷</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -857,7 +877,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.5" customWidth="1"/>
@@ -1070,6 +1090,38 @@
         <v>94</v>
       </c>
     </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" t="s">
+        <v>64</v>
+      </c>
+      <c r="I8" t="s">
+        <v>92</v>
+      </c>
+      <c r="J8" t="s">
+        <v>81</v>
+      </c>
+    </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>8</v>
@@ -1294,16 +1346,22 @@
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="D21" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E21" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="F21" t="s">
-        <v>63</v>
+        <v>74</v>
+      </c>
+      <c r="G21" t="s">
+        <v>127</v>
+      </c>
+      <c r="H21" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.45">
@@ -1314,59 +1372,47 @@
         <v>3</v>
       </c>
       <c r="C22" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D22" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="E22" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="F22" t="s">
-        <v>74</v>
-      </c>
-      <c r="G22" t="s">
-        <v>117</v>
-      </c>
-      <c r="H22" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>122</v>
       </c>
       <c r="D23" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="E23" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="F23" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G23" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="H23" t="s">
-        <v>82</v>
-      </c>
-      <c r="I23" t="s">
-        <v>92</v>
-      </c>
-      <c r="J23" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" t="s">
         <v>3</v>
@@ -1375,44 +1421,56 @@
         <v>84</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E24" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="F24" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
       <c r="G24" t="s">
         <v>92</v>
       </c>
       <c r="H24" t="s">
+        <v>82</v>
+      </c>
+      <c r="I24" t="s">
+        <v>92</v>
+      </c>
+      <c r="J24" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B25" t="s">
         <v>3</v>
       </c>
       <c r="C25" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D25" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
         <v>92</v>
       </c>
-      <c r="F25" t="s">
+      <c r="H25" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
         <v>3</v>
@@ -1421,30 +1479,12 @@
         <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E26" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="F26" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" t="s">
-        <v>47</v>
-      </c>
-      <c r="H26" t="s">
-        <v>1</v>
-      </c>
-      <c r="I26" t="s">
-        <v>47</v>
-      </c>
-      <c r="J26" t="s">
-        <v>63</v>
-      </c>
-      <c r="K26" t="s">
-        <v>92</v>
-      </c>
-      <c r="L26" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1456,10 +1496,10 @@
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>105</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="E27" t="s">
         <v>47</v>
@@ -1473,30 +1513,48 @@
       <c r="H27" t="s">
         <v>1</v>
       </c>
+      <c r="I27" t="s">
+        <v>47</v>
+      </c>
+      <c r="J27" t="s">
+        <v>63</v>
+      </c>
+      <c r="K27" t="s">
+        <v>92</v>
+      </c>
+      <c r="L27" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D28" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E28" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="F28" t="s">
-        <v>64</v>
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>47</v>
+      </c>
+      <c r="H28" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29" t="s">
         <v>3</v>
@@ -1505,18 +1563,12 @@
         <v>108</v>
       </c>
       <c r="D29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E29" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="F29" t="s">
-        <v>14</v>
-      </c>
-      <c r="G29" t="s">
-        <v>92</v>
-      </c>
-      <c r="H29" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1528,33 +1580,59 @@
         <v>3</v>
       </c>
       <c r="C30" t="s">
+        <v>108</v>
+      </c>
+      <c r="D30" t="s">
+        <v>110</v>
+      </c>
+      <c r="E30" t="s">
+        <v>47</v>
+      </c>
+      <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>92</v>
+      </c>
+      <c r="H30" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
         <v>124</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D31" t="s">
         <v>126</v>
       </c>
-      <c r="E30" t="s">
-        <v>47</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="E31" t="s">
+        <v>47</v>
+      </c>
+      <c r="F31" t="s">
         <v>1</v>
       </c>
-      <c r="G30" t="s">
-        <v>47</v>
-      </c>
-      <c r="H30" t="s">
+      <c r="G31" t="s">
+        <v>47</v>
+      </c>
+      <c r="H31" t="s">
         <v>63</v>
       </c>
-      <c r="I30" t="s">
+      <c r="I31" t="s">
         <v>92</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J31" t="s">
         <v>64</v>
       </c>
-      <c r="K30" t="s">
+      <c r="K31" t="s">
         <v>92</v>
       </c>
-      <c r="L30" t="s">
+      <c r="L31" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1566,7 +1644,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3095CB9C-57DF-42C7-A3A3-0F6AEE65EA25}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
@@ -1754,6 +1832,20 @@
       </c>
       <c r="D15" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D16" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>